<commit_message>
Remote Sensor Client BOM Battery Link added
</commit_message>
<xml_diff>
--- a/Design Files/Remote_Sensor_Unit/BOM/Client_BOM_Remote_Sensor_Unit.xlsx
+++ b/Design Files/Remote_Sensor_Unit/BOM/Client_BOM_Remote_Sensor_Unit.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="619" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="620" uniqueCount="417">
   <si>
     <t>Component list</t>
   </si>
@@ -1833,6 +1833,9 @@
     <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1841,9 +1844,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2213,10 +2213,10 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="63"/>
-      <c r="L1" s="63"/>
+      <c r="I1" s="64"/>
+      <c r="J1" s="64"/>
+      <c r="K1" s="64"/>
+      <c r="L1" s="64"/>
     </row>
     <row r="2" spans="1:12" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2252,7 +2252,7 @@
       <c r="I3" s="4"/>
       <c r="J3" s="4"/>
       <c r="K3" s="4"/>
-      <c r="L3" s="64"/>
+      <c r="L3" s="65"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2270,7 +2270,7 @@
       <c r="I4" s="6"/>
       <c r="J4" s="6"/>
       <c r="K4" s="6"/>
-      <c r="L4" s="65"/>
+      <c r="L4" s="66"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -2288,7 +2288,7 @@
       <c r="I5" s="5"/>
       <c r="J5" s="5"/>
       <c r="K5" s="5"/>
-      <c r="L5" s="65"/>
+      <c r="L5" s="66"/>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -2302,7 +2302,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
       <c r="K6" s="5"/>
-      <c r="L6" s="65"/>
+      <c r="L6" s="66"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -2316,7 +2316,7 @@
       <c r="I7" s="7"/>
       <c r="J7" s="7"/>
       <c r="K7" s="7"/>
-      <c r="L7" s="65"/>
+      <c r="L7" s="66"/>
     </row>
     <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -2330,7 +2330,7 @@
       <c r="I8" s="7"/>
       <c r="J8" s="7"/>
       <c r="K8" s="7"/>
-      <c r="L8" s="65"/>
+      <c r="L8" s="66"/>
     </row>
     <row r="9" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -5345,7 +5345,9 @@
         <f t="shared" si="41"/>
         <v>5</v>
       </c>
-      <c r="L92" s="38"/>
+      <c r="L92" s="63" t="s">
+        <v>412</v>
+      </c>
     </row>
     <row r="93" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
@@ -5380,7 +5382,7 @@
         <f t="shared" si="41"/>
         <v>5</v>
       </c>
-      <c r="L93" s="66" t="s">
+      <c r="L93" s="63" t="s">
         <v>412</v>
       </c>
     </row>
@@ -5417,7 +5419,7 @@
         <f t="shared" si="41"/>
         <v>5</v>
       </c>
-      <c r="L94" s="66" t="s">
+      <c r="L94" s="63" t="s">
         <v>412</v>
       </c>
     </row>
@@ -5492,9 +5494,10 @@
   <hyperlinks>
     <hyperlink ref="L93" r:id="rId1"/>
     <hyperlink ref="L94" r:id="rId2"/>
+    <hyperlink ref="L92" r:id="rId3"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId3"/>
-  <drawing r:id="rId4"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId4"/>
+  <drawing r:id="rId5"/>
 </worksheet>
 </file>
</xml_diff>